<commit_message>
feat(scrapers/sites): +7 gestora extractors — 21 ISIN + 13 min_subs auto
Adiciona extractors para BlueCrow, GNB, Optimize, Sixty Degrees, CGD,
Banco BPI, Banco Invest (Smart Invest). Unescape HTML entities no _get
(sites.bancobpi.pt / .gnbga.pt / .bluecrowcapital.com usam &ccedil;&atilde;)
e normaliza formato numérico pt-PT (1.000,50) via helper _num.

Cobertura subiu:
- ISIN:     6 → 21 fundos
- min_subs: 10 → 13 fundos

URLs wired em MANUAL_OVERRIDES (universe.py):
- BlueCrow Global Opportunities, Caixa ALG, GNB (2 fichas),
  Optimize (4 PPRs), Sixty Degrees (3 famílias), Smart Invest hub,
  BPI Global Equities, Oxy Capital public-markets (52 categorias).

Notas:
- BPI não expõe ISIN em HTML (injectado por JS) — só Global Equities
  foi wired mas não extrai campos.
- Caixa Wealth pages são SPA, ISIN só aparece em fichas PDF — fica
  por automatizar.
- Sixty PPR/OICVM Flexível extrai ISIN errado (partilha página com
  Ações Globais). Precisa de URL específico por categoria.
</commit_message>
<xml_diff>
--- a/data/ppr_status.xlsx
+++ b/data/ppr_status.xlsx
@@ -2942,8 +2942,14 @@
         <v>0.02</v>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>PTBLWTHM0004</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>1000</v>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -2986,7 +2992,11 @@
         <v>1.81</v>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>PTIXAEHM0006</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
@@ -3854,8 +3864,14 @@
       <c r="I54" t="n">
         <v>4</v>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>PTYESALM0007</t>
+        </is>
+      </c>
+      <c r="K54" t="n">
+        <v>25</v>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA HARMONIZADOS</t>
@@ -3896,8 +3912,14 @@
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>PTGNFHHM0002</t>
+        </is>
+      </c>
+      <c r="K55" t="n">
+        <v>5</v>
+      </c>
       <c r="L55" t="inlineStr">
         <is>
           <t>FUNDOS DE AÇÕES DE FUNDOS POUPANÇA-REFORMA HARMONIZADOS</t>
@@ -4272,7 +4294,11 @@
       <c r="I63" t="n">
         <v>5</v>
       </c>
-      <c r="J63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>PTOPZEHM0017</t>
+        </is>
+      </c>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
@@ -4318,7 +4344,11 @@
       <c r="I64" t="n">
         <v>4</v>
       </c>
-      <c r="J64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>PTOPZAHM0003</t>
+        </is>
+      </c>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
@@ -4364,7 +4394,11 @@
       <c r="I65" t="n">
         <v>4</v>
       </c>
-      <c r="J65" t="inlineStr"/>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>PTOPZBHM0002</t>
+        </is>
+      </c>
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
@@ -4410,7 +4444,11 @@
       <c r="I66" t="n">
         <v>4</v>
       </c>
-      <c r="J66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>PTOPZDHM0000</t>
+        </is>
+      </c>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
@@ -6618,7 +6656,11 @@
       <c r="I115" t="n">
         <v>3</v>
       </c>
-      <c r="J115" t="inlineStr"/>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>PTSXYXHM0003</t>
+        </is>
+      </c>
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
@@ -6664,7 +6706,11 @@
       <c r="I116" t="n">
         <v>3</v>
       </c>
-      <c r="J116" t="inlineStr"/>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>PTSXYAHM0000</t>
+        </is>
+      </c>
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
@@ -6710,7 +6756,11 @@
       <c r="I117" t="n">
         <v>3</v>
       </c>
-      <c r="J117" t="inlineStr"/>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>PTSXYAHM0000</t>
+        </is>
+      </c>
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
@@ -6756,7 +6806,11 @@
       <c r="I118" t="n">
         <v>3</v>
       </c>
-      <c r="J118" t="inlineStr"/>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>PTSXYAHM0000</t>
+        </is>
+      </c>
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
@@ -6802,7 +6856,11 @@
       <c r="I119" t="n">
         <v>4</v>
       </c>
-      <c r="J119" t="inlineStr"/>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>PTARMIHM0004</t>
+        </is>
+      </c>
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
@@ -6848,7 +6906,11 @@
       <c r="I120" t="n">
         <v>4</v>
       </c>
-      <c r="J120" t="inlineStr"/>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>PTARMIHM0004</t>
+        </is>
+      </c>
       <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
@@ -6894,7 +6956,11 @@
       <c r="I121" t="n">
         <v>4</v>
       </c>
-      <c r="J121" t="inlineStr"/>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>PTARMIHM0004</t>
+        </is>
+      </c>
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
@@ -8680,8 +8746,14 @@
         <v>0.02</v>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>PTBLWTHM0004</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>1000</v>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -8724,7 +8796,11 @@
         <v>1.81</v>
       </c>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>PTIXAEHM0006</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
@@ -9700,8 +9776,14 @@
       <c r="I57" t="n">
         <v>4</v>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>PTYESALM0007</t>
+        </is>
+      </c>
+      <c r="K57" t="n">
+        <v>25</v>
+      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA HARMONIZADOS</t>
@@ -9742,8 +9824,14 @@
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>PTGNFHHM0002</t>
+        </is>
+      </c>
+      <c r="K58" t="n">
+        <v>5</v>
+      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>FUNDOS DE AÇÕES DE FUNDOS POUPANÇA-REFORMA HARMONIZADOS</t>
@@ -10622,7 +10710,11 @@
       <c r="I78" t="n">
         <v>5</v>
       </c>
-      <c r="J78" t="inlineStr"/>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>PTOPZEHM0017</t>
+        </is>
+      </c>
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
@@ -10668,7 +10760,11 @@
       <c r="I79" t="n">
         <v>4</v>
       </c>
-      <c r="J79" t="inlineStr"/>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>PTOPZAHM0003</t>
+        </is>
+      </c>
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
@@ -10714,7 +10810,11 @@
       <c r="I80" t="n">
         <v>4</v>
       </c>
-      <c r="J80" t="inlineStr"/>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>PTOPZBHM0002</t>
+        </is>
+      </c>
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
@@ -10760,7 +10860,11 @@
       <c r="I81" t="n">
         <v>4</v>
       </c>
-      <c r="J81" t="inlineStr"/>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>PTOPZDHM0000</t>
+        </is>
+      </c>
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
@@ -13178,7 +13282,11 @@
       <c r="I135" t="n">
         <v>3</v>
       </c>
-      <c r="J135" t="inlineStr"/>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>PTSXYXHM0003</t>
+        </is>
+      </c>
       <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr">
         <is>
@@ -13224,7 +13332,11 @@
       <c r="I136" t="n">
         <v>3</v>
       </c>
-      <c r="J136" t="inlineStr"/>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>PTSXYAHM0000</t>
+        </is>
+      </c>
       <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr">
         <is>
@@ -13270,7 +13382,11 @@
       <c r="I137" t="n">
         <v>3</v>
       </c>
-      <c r="J137" t="inlineStr"/>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>PTSXYAHM0000</t>
+        </is>
+      </c>
       <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr">
         <is>
@@ -13316,7 +13432,11 @@
       <c r="I138" t="n">
         <v>3</v>
       </c>
-      <c r="J138" t="inlineStr"/>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>PTSXYAHM0000</t>
+        </is>
+      </c>
       <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr">
         <is>
@@ -13362,7 +13482,11 @@
       <c r="I139" t="n">
         <v>4</v>
       </c>
-      <c r="J139" t="inlineStr"/>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>PTARMIHM0004</t>
+        </is>
+      </c>
       <c r="K139" t="inlineStr"/>
       <c r="L139" t="inlineStr">
         <is>
@@ -13408,7 +13532,11 @@
       <c r="I140" t="n">
         <v>4</v>
       </c>
-      <c r="J140" t="inlineStr"/>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>PTARMIHM0004</t>
+        </is>
+      </c>
       <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr">
         <is>
@@ -13454,7 +13582,11 @@
       <c r="I141" t="n">
         <v>4</v>
       </c>
-      <c r="J141" t="inlineStr"/>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>PTARMIHM0004</t>
+        </is>
+      </c>
       <c r="K141" t="inlineStr"/>
       <c r="L141" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: PDF IFIs + Santander/Bankinter/Optimize Leopardo/SGF ISINs
- Add pypdf dependency + _get_pdf_text helper for parsing IFI PDFs.
- extract_cgd_pdf: extracts ISIN + TEC from Caixa IFI PDFs (4 Wealth
  PDFs wired → 4 Wealth sub-families get ISIN/TEC).
- extract_sgf_pdf: parses Golden SGF Doc-Informativo PDFs (single and
  multi-class). URL can be .pdf directly.
- extract_santander: HTML extractor for santander.pt fund pages.
- Hardcode Optimize LFO Leopardo 3 categorias (ISIN + min_subs + TEC
  from attached IFI PDF: Premium 500k€/1.11%, Discount 10k€/2.19%,
  Standard 1k€/2.47%).
- Hardcode Golden SGF ETF Plus/Start (ISIN + min_subs + comissão
  gestão as TEC approximation, from user-attached PDF).
- Map 10 other SGF funds to their ISINs by cross-referencing PDF
  authorization dates against Excel first-price dates.
- Wire Bankinter 25/50/75/100, Santander (3), Caixa Wealth (4 PDFs),
  BPI Global Equities.

Coverage delta:
- ISIN:     21 → 66 funds
- min_subs: 13 → 18 funds
</commit_message>
<xml_diff>
--- a/data/ppr_status.xlsx
+++ b/data/ppr_status.xlsx
@@ -678,10 +678,18 @@
           <t>2025-11-06</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>0.75</v>
+      </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>PTFP00000762</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>10000</v>
+      </c>
       <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -720,10 +728,18 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>PTFP00000861</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>1500</v>
+      </c>
       <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -764,7 +780,11 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>PTFP00000416</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
     </row>
@@ -806,7 +826,11 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>PTFP00000424</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
     </row>
@@ -848,7 +872,11 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>PTFP00000382</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
     </row>
@@ -890,7 +918,11 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>PTFP00000432</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
     </row>
@@ -974,7 +1006,11 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>PTFP00000515</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
     </row>
@@ -1016,7 +1052,11 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>PTFP00000879</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
     </row>
@@ -1058,7 +1098,11 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>PTFP00000507</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
     </row>
@@ -1100,7 +1144,11 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>PTFP00000473</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
     </row>
@@ -1184,7 +1232,11 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>PTFP00000390</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
     </row>
@@ -1268,7 +1320,11 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>PTFP00000770</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
     </row>
@@ -2034,7 +2090,11 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
@@ -2076,7 +2136,11 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
@@ -2118,7 +2182,11 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
@@ -2164,7 +2232,11 @@
       <c r="I17" t="n">
         <v>4</v>
       </c>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
@@ -2210,7 +2282,11 @@
       <c r="I18" t="n">
         <v>4</v>
       </c>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
@@ -2256,7 +2332,11 @@
       <c r="I19" t="n">
         <v>4</v>
       </c>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
@@ -2302,7 +2382,11 @@
       <c r="I20" t="n">
         <v>4</v>
       </c>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>PTYBCFHM0017</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
@@ -2348,7 +2432,11 @@
       <c r="I21" t="n">
         <v>4</v>
       </c>
-      <c r="J21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>PTYBCFHM0017</t>
+        </is>
+      </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
@@ -2394,7 +2482,11 @@
       <c r="I22" t="n">
         <v>4</v>
       </c>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>PTYBCFHM0017</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
@@ -2440,7 +2532,11 @@
       <c r="I23" t="n">
         <v>5</v>
       </c>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>PTYBCQLM0000</t>
+        </is>
+      </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
@@ -2486,7 +2582,11 @@
       <c r="I24" t="n">
         <v>5</v>
       </c>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>PTYBCQLM0000</t>
+        </is>
+      </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
@@ -2532,7 +2632,11 @@
       <c r="I25" t="n">
         <v>5</v>
       </c>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>PTYBCQLM0000</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
@@ -3042,7 +3146,11 @@
       <c r="I36" t="n">
         <v>5</v>
       </c>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>PTCXGBHM0017</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
@@ -3088,7 +3196,11 @@
       <c r="I37" t="n">
         <v>5</v>
       </c>
-      <c r="J37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>PTCXGBHM0017</t>
+        </is>
+      </c>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
@@ -3134,7 +3246,11 @@
       <c r="I38" t="n">
         <v>5</v>
       </c>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>PTCXGBHM0017</t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
@@ -3180,7 +3296,11 @@
       <c r="I39" t="n">
         <v>5</v>
       </c>
-      <c r="J39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>PTCXGBHM0017</t>
+        </is>
+      </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
@@ -3224,7 +3344,11 @@
         <v>1.83</v>
       </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>PTCXGWHM0020</t>
+        </is>
+      </c>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
@@ -3268,7 +3392,11 @@
         <v>1.68</v>
       </c>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>PTCXGWHM0020</t>
+        </is>
+      </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
@@ -3312,7 +3440,11 @@
         <v>1.47</v>
       </c>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>PTCXGWHM0020</t>
+        </is>
+      </c>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
@@ -3358,7 +3490,11 @@
       <c r="I43" t="n">
         <v>4</v>
       </c>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>PTIXAFHM0005</t>
+        </is>
+      </c>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
@@ -3404,7 +3540,11 @@
       <c r="I44" t="n">
         <v>4</v>
       </c>
-      <c r="J44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>PTIXAFHM0005</t>
+        </is>
+      </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
@@ -3450,7 +3590,11 @@
       <c r="I45" t="n">
         <v>4</v>
       </c>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>PTIXAFHM0005</t>
+        </is>
+      </c>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
@@ -3496,7 +3640,11 @@
       <c r="I46" t="n">
         <v>4</v>
       </c>
-      <c r="J46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>PTIXAFHM0005</t>
+        </is>
+      </c>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
@@ -3542,7 +3690,11 @@
       <c r="I47" t="n">
         <v>4</v>
       </c>
-      <c r="J47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>PTCXGMHM0014</t>
+        </is>
+      </c>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
@@ -3588,7 +3740,11 @@
       <c r="I48" t="n">
         <v>4</v>
       </c>
-      <c r="J48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>PTCXGMHM0014</t>
+        </is>
+      </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
@@ -3634,7 +3790,11 @@
       <c r="I49" t="n">
         <v>4</v>
       </c>
-      <c r="J49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>PTCXGMHM0014</t>
+        </is>
+      </c>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
@@ -3680,7 +3840,11 @@
       <c r="I50" t="n">
         <v>4</v>
       </c>
-      <c r="J50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>PTCXGMHM0014</t>
+        </is>
+      </c>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
@@ -6518,8 +6682,14 @@
       <c r="I112" t="n">
         <v>5</v>
       </c>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>PTOPZUHM0009</t>
+        </is>
+      </c>
+      <c r="K112" t="n">
+        <v>10000</v>
+      </c>
       <c r="L112" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA HARMONIZADOS</t>
@@ -6564,8 +6734,14 @@
       <c r="I113" t="n">
         <v>5</v>
       </c>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>PTOPZQHM0005</t>
+        </is>
+      </c>
+      <c r="K113" t="n">
+        <v>500000</v>
+      </c>
       <c r="L113" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA HARMONIZADOS</t>
@@ -6610,8 +6786,14 @@
       <c r="I114" t="n">
         <v>5</v>
       </c>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>PTOPZVHM0008</t>
+        </is>
+      </c>
+      <c r="K114" t="n">
+        <v>1000</v>
+      </c>
       <c r="L114" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA HARMONIZADOS</t>
@@ -7006,7 +7188,11 @@
       <c r="I122" t="n">
         <v>3</v>
       </c>
-      <c r="J122" t="inlineStr"/>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>PTSFFAHM0013</t>
+        </is>
+      </c>
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
@@ -7052,7 +7238,11 @@
       <c r="I123" t="n">
         <v>3</v>
       </c>
-      <c r="J123" t="inlineStr"/>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>PTYSAVLM0006</t>
+        </is>
+      </c>
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
@@ -7098,7 +7288,11 @@
       <c r="I124" t="n">
         <v>3</v>
       </c>
-      <c r="J124" t="inlineStr"/>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>PTYMCRLM0006</t>
+        </is>
+      </c>
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
@@ -7838,7 +8032,11 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
@@ -7880,7 +8078,11 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
@@ -7922,7 +8124,11 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
@@ -7968,7 +8174,11 @@
       <c r="I18" t="n">
         <v>4</v>
       </c>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
@@ -8014,7 +8224,11 @@
       <c r="I19" t="n">
         <v>4</v>
       </c>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
@@ -8060,7 +8274,11 @@
       <c r="I20" t="n">
         <v>4</v>
       </c>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>PTYBCPLM0001</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
@@ -8106,7 +8324,11 @@
       <c r="I21" t="n">
         <v>4</v>
       </c>
-      <c r="J21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>PTYBCFHM0017</t>
+        </is>
+      </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
@@ -8152,7 +8374,11 @@
       <c r="I22" t="n">
         <v>4</v>
       </c>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>PTYBCFHM0017</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
@@ -8198,7 +8424,11 @@
       <c r="I23" t="n">
         <v>4</v>
       </c>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>PTYBCFHM0017</t>
+        </is>
+      </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
@@ -8244,7 +8474,11 @@
       <c r="I24" t="n">
         <v>5</v>
       </c>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>PTYBCQLM0000</t>
+        </is>
+      </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
@@ -8290,7 +8524,11 @@
       <c r="I25" t="n">
         <v>5</v>
       </c>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>PTYBCQLM0000</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
@@ -8336,7 +8574,11 @@
       <c r="I26" t="n">
         <v>5</v>
       </c>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>PTYBCQLM0000</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
@@ -8846,7 +9088,11 @@
       <c r="I37" t="n">
         <v>5</v>
       </c>
-      <c r="J37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>PTCXGBHM0017</t>
+        </is>
+      </c>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
@@ -8892,7 +9138,11 @@
       <c r="I38" t="n">
         <v>5</v>
       </c>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>PTCXGBHM0017</t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
@@ -8938,7 +9188,11 @@
       <c r="I39" t="n">
         <v>5</v>
       </c>
-      <c r="J39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>PTCXGBHM0017</t>
+        </is>
+      </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
@@ -8984,7 +9238,11 @@
       <c r="I40" t="n">
         <v>5</v>
       </c>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>PTCXGBHM0017</t>
+        </is>
+      </c>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
@@ -9028,7 +9286,11 @@
         <v>1.83</v>
       </c>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>PTCXGWHM0020</t>
+        </is>
+      </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
@@ -9072,7 +9334,11 @@
         <v>1.68</v>
       </c>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>PTCXGWHM0020</t>
+        </is>
+      </c>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
@@ -9116,7 +9382,11 @@
         <v>1.47</v>
       </c>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>PTCXGWHM0020</t>
+        </is>
+      </c>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
@@ -9162,7 +9432,11 @@
       <c r="I44" t="n">
         <v>4</v>
       </c>
-      <c r="J44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>PTIXAFHM0005</t>
+        </is>
+      </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
@@ -9208,7 +9482,11 @@
       <c r="I45" t="n">
         <v>4</v>
       </c>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>PTIXAFHM0005</t>
+        </is>
+      </c>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
@@ -9254,7 +9532,11 @@
       <c r="I46" t="n">
         <v>4</v>
       </c>
-      <c r="J46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>PTIXAFHM0005</t>
+        </is>
+      </c>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
@@ -9300,7 +9582,11 @@
       <c r="I47" t="n">
         <v>4</v>
       </c>
-      <c r="J47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>PTIXAFHM0005</t>
+        </is>
+      </c>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
@@ -9346,7 +9632,11 @@
       <c r="I48" t="n">
         <v>4</v>
       </c>
-      <c r="J48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>PTCXGMHM0014</t>
+        </is>
+      </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
@@ -9392,7 +9682,11 @@
       <c r="I49" t="n">
         <v>4</v>
       </c>
-      <c r="J49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>PTCXGMHM0014</t>
+        </is>
+      </c>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
@@ -9438,7 +9732,11 @@
       <c r="I50" t="n">
         <v>4</v>
       </c>
-      <c r="J50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>PTCXGMHM0014</t>
+        </is>
+      </c>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
@@ -9484,7 +9782,11 @@
       <c r="I51" t="n">
         <v>4</v>
       </c>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>PTCXGMHM0014</t>
+        </is>
+      </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
@@ -9874,10 +10176,18 @@
           <t>2025-11-06</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
+      <c r="H59" t="n">
+        <v>0.75</v>
+      </c>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>PTFP00000762</t>
+        </is>
+      </c>
+      <c r="K59" t="n">
+        <v>10000</v>
+      </c>
       <c r="L59" t="inlineStr"/>
     </row>
     <row r="60">
@@ -9916,10 +10226,18 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" t="n">
+        <v>1</v>
+      </c>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>PTFP00000861</t>
+        </is>
+      </c>
+      <c r="K60" t="n">
+        <v>1500</v>
+      </c>
       <c r="L60" t="inlineStr"/>
     </row>
     <row r="61">
@@ -9960,7 +10278,11 @@
       </c>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>PTFP00000416</t>
+        </is>
+      </c>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>
     </row>
@@ -10002,7 +10324,11 @@
       </c>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>PTFP00000424</t>
+        </is>
+      </c>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr"/>
     </row>
@@ -10044,7 +10370,11 @@
       </c>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>PTFP00000382</t>
+        </is>
+      </c>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr"/>
     </row>
@@ -10086,7 +10416,11 @@
       </c>
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>PTFP00000432</t>
+        </is>
+      </c>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr"/>
     </row>
@@ -10170,7 +10504,11 @@
       </c>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>PTFP00000515</t>
+        </is>
+      </c>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr"/>
     </row>
@@ -10212,7 +10550,11 @@
       </c>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>PTFP00000879</t>
+        </is>
+      </c>
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr"/>
     </row>
@@ -10254,7 +10596,11 @@
       </c>
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>PTFP00000507</t>
+        </is>
+      </c>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
     </row>
@@ -10296,7 +10642,11 @@
       </c>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>PTFP00000473</t>
+        </is>
+      </c>
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr"/>
     </row>
@@ -12934,8 +13284,14 @@
       <c r="I127" t="n">
         <v>5</v>
       </c>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>PTOPZUHM0009</t>
+        </is>
+      </c>
+      <c r="K127" t="n">
+        <v>10000</v>
+      </c>
       <c r="L127" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA HARMONIZADOS</t>
@@ -12980,8 +13336,14 @@
       <c r="I128" t="n">
         <v>5</v>
       </c>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>PTOPZQHM0005</t>
+        </is>
+      </c>
+      <c r="K128" t="n">
+        <v>500000</v>
+      </c>
       <c r="L128" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA HARMONIZADOS</t>
@@ -13026,8 +13388,14 @@
       <c r="I129" t="n">
         <v>5</v>
       </c>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>PTOPZVHM0008</t>
+        </is>
+      </c>
+      <c r="K129" t="n">
+        <v>1000</v>
+      </c>
       <c r="L129" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA HARMONIZADOS</t>
@@ -13072,7 +13440,11 @@
       </c>
       <c r="H130" t="inlineStr"/>
       <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>PTFP00000390</t>
+        </is>
+      </c>
       <c r="K130" t="inlineStr"/>
       <c r="L130" t="inlineStr"/>
     </row>
@@ -13156,7 +13528,11 @@
       </c>
       <c r="H132" t="inlineStr"/>
       <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>PTFP00000770</t>
+        </is>
+      </c>
       <c r="K132" t="inlineStr"/>
       <c r="L132" t="inlineStr"/>
     </row>
@@ -13632,7 +14008,11 @@
       <c r="I142" t="n">
         <v>3</v>
       </c>
-      <c r="J142" t="inlineStr"/>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>PTSFFAHM0013</t>
+        </is>
+      </c>
       <c r="K142" t="inlineStr"/>
       <c r="L142" t="inlineStr">
         <is>
@@ -13678,7 +14058,11 @@
       <c r="I143" t="n">
         <v>3</v>
       </c>
-      <c r="J143" t="inlineStr"/>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>PTYSAVLM0006</t>
+        </is>
+      </c>
       <c r="K143" t="inlineStr"/>
       <c r="L143" t="inlineStr">
         <is>
@@ -13724,7 +14108,11 @@
       <c r="I144" t="n">
         <v>3</v>
       </c>
-      <c r="J144" t="inlineStr"/>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>PTYMCRLM0006</t>
+        </is>
+      </c>
       <c r="K144" t="inlineStr"/>
       <c r="L144" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: Oxy Capital — ISIN+TEC+min_subs para 48 categorias (via IFI PDF)
O IFI da Oxy Capital Liquid Opportunities lista explicitamente os 53
códigos ISIN por categoria (AA, BA-BL, CA, DA-DI, EA-EL, FA-FS).
Destas, 48 existem no universo CMVM.

- Tabela _OXY_MAP em universe.py com (ISIN, min_subs, TEC) por cat.
- Loop gera 48 overrides a partir da tabela.
- Grupos:
  · A/C:  sem min, TEC 0.16% (>€15M AuM)
  · B/D:  €100k (colaboradores), TEC 0.76%
  · E:    sem min, TEC 0.56%
  · F:    €2.000,  TEC 1.06%
- PDF tem BH-BL e DI que não estão no CMVM (futuras?);
  CMVM tem EM/EN/EO que não estão no PDF desta revisão.

Coverage:
  ISIN:     66 → 110 funds
  min_subs: 18 → 48 funds
</commit_message>
<xml_diff>
--- a/data/ppr_status.xlsx
+++ b/data/ppr_status.xlsx
@@ -4653,12 +4653,16 @@
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>0.26</v>
+        <v>0.16</v>
       </c>
       <c r="I67" t="n">
         <v>4</v>
       </c>
-      <c r="J67" t="inlineStr"/>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>PTOXCRHM0001</t>
+        </is>
+      </c>
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
@@ -4699,13 +4703,19 @@
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I68" t="n">
         <v>4</v>
       </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>PTOXCSHM0000</t>
+        </is>
+      </c>
+      <c r="K68" t="n">
+        <v>100000</v>
+      </c>
       <c r="L68" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -4745,13 +4755,19 @@
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I69" t="n">
         <v>4</v>
       </c>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>PTOYAAHM0001</t>
+        </is>
+      </c>
+      <c r="K69" t="n">
+        <v>100000</v>
+      </c>
       <c r="L69" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -4791,13 +4807,19 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I70" t="n">
         <v>4</v>
       </c>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>PTOYABHM0000</t>
+        </is>
+      </c>
+      <c r="K70" t="n">
+        <v>100000</v>
+      </c>
       <c r="L70" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -4837,13 +4859,19 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I71" t="n">
         <v>4</v>
       </c>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>PTOYACHM0009</t>
+        </is>
+      </c>
+      <c r="K71" t="n">
+        <v>100000</v>
+      </c>
       <c r="L71" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -4883,13 +4911,19 @@
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I72" t="n">
         <v>4</v>
       </c>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>PTOYADHM0008</t>
+        </is>
+      </c>
+      <c r="K72" t="n">
+        <v>100000</v>
+      </c>
       <c r="L72" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -4929,13 +4963,19 @@
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I73" t="n">
         <v>4</v>
       </c>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>PTOYAEHM0007</t>
+        </is>
+      </c>
+      <c r="K73" t="n">
+        <v>100000</v>
+      </c>
       <c r="L73" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -4974,12 +5014,20 @@
         </is>
       </c>
       <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
+      <c r="H74" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I74" t="n">
         <v>4</v>
       </c>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>PTOYAFHM0006</t>
+        </is>
+      </c>
+      <c r="K74" t="n">
+        <v>100000</v>
+      </c>
       <c r="L74" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -5019,12 +5067,16 @@
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>0.26</v>
+        <v>0.16</v>
       </c>
       <c r="I75" t="n">
         <v>4</v>
       </c>
-      <c r="J75" t="inlineStr"/>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>PTOXCTHM0009</t>
+        </is>
+      </c>
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
@@ -5065,13 +5117,19 @@
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I76" t="n">
         <v>4</v>
       </c>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>PTOXCUHM0006</t>
+        </is>
+      </c>
+      <c r="K76" t="n">
+        <v>100000</v>
+      </c>
       <c r="L76" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -5110,12 +5168,20 @@
         </is>
       </c>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
+      <c r="H77" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I77" t="n">
         <v>4</v>
       </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>PTOYAIHM0003</t>
+        </is>
+      </c>
+      <c r="K77" t="n">
+        <v>100000</v>
+      </c>
       <c r="L77" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -5154,12 +5220,20 @@
         </is>
       </c>
       <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
+      <c r="H78" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I78" t="n">
         <v>4</v>
       </c>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>PTOYAJHM0002</t>
+        </is>
+      </c>
+      <c r="K78" t="n">
+        <v>100000</v>
+      </c>
       <c r="L78" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -5198,12 +5272,20 @@
         </is>
       </c>
       <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
+      <c r="H79" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I79" t="n">
         <v>4</v>
       </c>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>PTOYAKHM0009</t>
+        </is>
+      </c>
+      <c r="K79" t="n">
+        <v>100000</v>
+      </c>
       <c r="L79" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -5242,12 +5324,20 @@
         </is>
       </c>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
+      <c r="H80" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I80" t="n">
         <v>4</v>
       </c>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>PTOYALHM0008</t>
+        </is>
+      </c>
+      <c r="K80" t="n">
+        <v>100000</v>
+      </c>
       <c r="L80" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -5286,12 +5376,20 @@
         </is>
       </c>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
+      <c r="H81" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I81" t="n">
         <v>4</v>
       </c>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>PTOYAMHM0007</t>
+        </is>
+      </c>
+      <c r="K81" t="n">
+        <v>100000</v>
+      </c>
       <c r="L81" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -5331,12 +5429,16 @@
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>0.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I82" t="n">
         <v>4</v>
       </c>
-      <c r="J82" t="inlineStr"/>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>PTOXTAHM0001</t>
+        </is>
+      </c>
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
@@ -5377,12 +5479,16 @@
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="n">
-        <v>0.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I83" t="n">
         <v>4</v>
       </c>
-      <c r="J83" t="inlineStr"/>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>PTOYAQHM0003</t>
+        </is>
+      </c>
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
@@ -5423,12 +5529,16 @@
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>0.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I84" t="n">
         <v>4</v>
       </c>
-      <c r="J84" t="inlineStr"/>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>PTOYARHM0002</t>
+        </is>
+      </c>
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
@@ -5469,12 +5579,16 @@
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>0.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I85" t="n">
         <v>4</v>
       </c>
-      <c r="J85" t="inlineStr"/>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>PTOYASHM0001</t>
+        </is>
+      </c>
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
@@ -5515,12 +5629,16 @@
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>0.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I86" t="n">
         <v>4</v>
       </c>
-      <c r="J86" t="inlineStr"/>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>PTOYATHM0000</t>
+        </is>
+      </c>
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
@@ -5560,11 +5678,17 @@
         </is>
       </c>
       <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
+      <c r="H87" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I87" t="n">
         <v>4</v>
       </c>
-      <c r="J87" t="inlineStr"/>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>PTOYAUHM0007</t>
+        </is>
+      </c>
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
@@ -5604,11 +5728,17 @@
         </is>
       </c>
       <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
+      <c r="H88" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I88" t="n">
         <v>4</v>
       </c>
-      <c r="J88" t="inlineStr"/>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>PTOYAVHM0006</t>
+        </is>
+      </c>
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
@@ -5648,11 +5778,17 @@
         </is>
       </c>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
+      <c r="H89" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I89" t="n">
         <v>4</v>
       </c>
-      <c r="J89" t="inlineStr"/>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>PTOYAWHM0005</t>
+        </is>
+      </c>
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
@@ -5692,11 +5828,17 @@
         </is>
       </c>
       <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
+      <c r="H90" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I90" t="n">
         <v>4</v>
       </c>
-      <c r="J90" t="inlineStr"/>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>PTOYAXHM0004</t>
+        </is>
+      </c>
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
@@ -5736,11 +5878,17 @@
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
+      <c r="H91" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I91" t="n">
         <v>4</v>
       </c>
-      <c r="J91" t="inlineStr"/>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>PTOXS3HM0000</t>
+        </is>
+      </c>
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
@@ -5780,11 +5928,17 @@
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
+      <c r="H92" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I92" t="n">
         <v>4</v>
       </c>
-      <c r="J92" t="inlineStr"/>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>PTOXS4HM0009</t>
+        </is>
+      </c>
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
@@ -5824,11 +5978,17 @@
         </is>
       </c>
       <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
+      <c r="H93" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I93" t="n">
         <v>4</v>
       </c>
-      <c r="J93" t="inlineStr"/>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>PTOXS5HM0008</t>
+        </is>
+      </c>
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
@@ -5913,13 +6073,19 @@
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I95" t="n">
         <v>4</v>
       </c>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>PTOXTBHM0000</t>
+        </is>
+      </c>
+      <c r="K95" t="n">
+        <v>2000</v>
+      </c>
       <c r="L95" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -5959,13 +6125,19 @@
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I96" t="n">
         <v>4</v>
       </c>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>PTOYAYHM0003</t>
+        </is>
+      </c>
+      <c r="K96" t="n">
+        <v>2000</v>
+      </c>
       <c r="L96" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6005,13 +6177,19 @@
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I97" t="n">
         <v>4</v>
       </c>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>PTOYAZHM0002</t>
+        </is>
+      </c>
+      <c r="K97" t="n">
+        <v>2000</v>
+      </c>
       <c r="L97" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6051,13 +6229,19 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I98" t="n">
         <v>4</v>
       </c>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>PTOYA1HM0008</t>
+        </is>
+      </c>
+      <c r="K98" t="n">
+        <v>2000</v>
+      </c>
       <c r="L98" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6097,13 +6281,19 @@
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I99" t="n">
         <v>4</v>
       </c>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>PTOYA2HM0007</t>
+        </is>
+      </c>
+      <c r="K99" t="n">
+        <v>2000</v>
+      </c>
       <c r="L99" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6143,13 +6333,19 @@
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I100" t="n">
         <v>4</v>
       </c>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>PTOYA3HM0006</t>
+        </is>
+      </c>
+      <c r="K100" t="n">
+        <v>2000</v>
+      </c>
       <c r="L100" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6189,13 +6385,19 @@
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I101" t="n">
         <v>4</v>
       </c>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>PTOYA4HM0005</t>
+        </is>
+      </c>
+      <c r="K101" t="n">
+        <v>2000</v>
+      </c>
       <c r="L101" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6235,13 +6437,19 @@
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I102" t="n">
         <v>4</v>
       </c>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>PTOYA5HM0004</t>
+        </is>
+      </c>
+      <c r="K102" t="n">
+        <v>2000</v>
+      </c>
       <c r="L102" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6280,12 +6488,20 @@
         </is>
       </c>
       <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
+      <c r="H103" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I103" t="n">
         <v>4</v>
       </c>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>PTOYA6HM0003</t>
+        </is>
+      </c>
+      <c r="K103" t="n">
+        <v>2000</v>
+      </c>
       <c r="L103" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6324,12 +6540,20 @@
         </is>
       </c>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
+      <c r="H104" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I104" t="n">
         <v>4</v>
       </c>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>PTOXSMHM0008</t>
+        </is>
+      </c>
+      <c r="K104" t="n">
+        <v>2000</v>
+      </c>
       <c r="L104" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6368,12 +6592,20 @@
         </is>
       </c>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
+      <c r="H105" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I105" t="n">
         <v>4</v>
       </c>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>PTOXSNHM0007</t>
+        </is>
+      </c>
+      <c r="K105" t="n">
+        <v>2000</v>
+      </c>
       <c r="L105" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6412,12 +6644,20 @@
         </is>
       </c>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
+      <c r="H106" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I106" t="n">
         <v>4</v>
       </c>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>PTOXSOHM0006</t>
+        </is>
+      </c>
+      <c r="K106" t="n">
+        <v>2000</v>
+      </c>
       <c r="L106" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6456,12 +6696,20 @@
         </is>
       </c>
       <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
+      <c r="H107" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I107" t="n">
         <v>4</v>
       </c>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>PTOXSPHM0005</t>
+        </is>
+      </c>
+      <c r="K107" t="n">
+        <v>2000</v>
+      </c>
       <c r="L107" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6500,12 +6748,20 @@
         </is>
       </c>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
+      <c r="H108" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I108" t="n">
         <v>4</v>
       </c>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>PTOXS6HM0007</t>
+        </is>
+      </c>
+      <c r="K108" t="n">
+        <v>2000</v>
+      </c>
       <c r="L108" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6544,12 +6800,20 @@
         </is>
       </c>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
+      <c r="H109" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I109" t="n">
         <v>4</v>
       </c>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>PTOXS7HM0006</t>
+        </is>
+      </c>
+      <c r="K109" t="n">
+        <v>2000</v>
+      </c>
       <c r="L109" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6588,12 +6852,20 @@
         </is>
       </c>
       <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
+      <c r="H110" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I110" t="n">
         <v>4</v>
       </c>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>PTOXS8HM0005</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>2000</v>
+      </c>
       <c r="L110" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -6632,12 +6904,20 @@
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
+      <c r="H111" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I111" t="n">
         <v>4</v>
       </c>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>PTOXS9HM0004</t>
+        </is>
+      </c>
+      <c r="K111" t="n">
+        <v>2000</v>
+      </c>
       <c r="L111" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11255,12 +11535,16 @@
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>0.26</v>
+        <v>0.16</v>
       </c>
       <c r="I82" t="n">
         <v>4</v>
       </c>
-      <c r="J82" t="inlineStr"/>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>PTOXCRHM0001</t>
+        </is>
+      </c>
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
@@ -11301,13 +11585,19 @@
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I83" t="n">
         <v>4</v>
       </c>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>PTOXCSHM0000</t>
+        </is>
+      </c>
+      <c r="K83" t="n">
+        <v>100000</v>
+      </c>
       <c r="L83" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11347,13 +11637,19 @@
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I84" t="n">
         <v>4</v>
       </c>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>PTOYAAHM0001</t>
+        </is>
+      </c>
+      <c r="K84" t="n">
+        <v>100000</v>
+      </c>
       <c r="L84" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11393,13 +11689,19 @@
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I85" t="n">
         <v>4</v>
       </c>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>PTOYABHM0000</t>
+        </is>
+      </c>
+      <c r="K85" t="n">
+        <v>100000</v>
+      </c>
       <c r="L85" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11439,13 +11741,19 @@
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I86" t="n">
         <v>4</v>
       </c>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>PTOYACHM0009</t>
+        </is>
+      </c>
+      <c r="K86" t="n">
+        <v>100000</v>
+      </c>
       <c r="L86" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11485,13 +11793,19 @@
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I87" t="n">
         <v>4</v>
       </c>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>PTOYADHM0008</t>
+        </is>
+      </c>
+      <c r="K87" t="n">
+        <v>100000</v>
+      </c>
       <c r="L87" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11531,13 +11845,19 @@
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I88" t="n">
         <v>4</v>
       </c>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>PTOYAEHM0007</t>
+        </is>
+      </c>
+      <c r="K88" t="n">
+        <v>100000</v>
+      </c>
       <c r="L88" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11576,12 +11896,20 @@
         </is>
       </c>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
+      <c r="H89" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I89" t="n">
         <v>4</v>
       </c>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>PTOYAFHM0006</t>
+        </is>
+      </c>
+      <c r="K89" t="n">
+        <v>100000</v>
+      </c>
       <c r="L89" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11621,12 +11949,16 @@
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>0.26</v>
+        <v>0.16</v>
       </c>
       <c r="I90" t="n">
         <v>4</v>
       </c>
-      <c r="J90" t="inlineStr"/>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>PTOXCTHM0009</t>
+        </is>
+      </c>
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
@@ -11667,13 +11999,19 @@
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>0.86</v>
+        <v>0.76</v>
       </c>
       <c r="I91" t="n">
         <v>4</v>
       </c>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>PTOXCUHM0006</t>
+        </is>
+      </c>
+      <c r="K91" t="n">
+        <v>100000</v>
+      </c>
       <c r="L91" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11712,12 +12050,20 @@
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
+      <c r="H92" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I92" t="n">
         <v>4</v>
       </c>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>PTOYAIHM0003</t>
+        </is>
+      </c>
+      <c r="K92" t="n">
+        <v>100000</v>
+      </c>
       <c r="L92" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11756,12 +12102,20 @@
         </is>
       </c>
       <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
+      <c r="H93" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I93" t="n">
         <v>4</v>
       </c>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>PTOYAJHM0002</t>
+        </is>
+      </c>
+      <c r="K93" t="n">
+        <v>100000</v>
+      </c>
       <c r="L93" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11800,12 +12154,20 @@
         </is>
       </c>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
+      <c r="H94" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I94" t="n">
         <v>4</v>
       </c>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>PTOYAKHM0009</t>
+        </is>
+      </c>
+      <c r="K94" t="n">
+        <v>100000</v>
+      </c>
       <c r="L94" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11844,12 +12206,20 @@
         </is>
       </c>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
+      <c r="H95" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I95" t="n">
         <v>4</v>
       </c>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>PTOYALHM0008</t>
+        </is>
+      </c>
+      <c r="K95" t="n">
+        <v>100000</v>
+      </c>
       <c r="L95" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11888,12 +12258,20 @@
         </is>
       </c>
       <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
+      <c r="H96" t="n">
+        <v>0.76</v>
+      </c>
       <c r="I96" t="n">
         <v>4</v>
       </c>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>PTOYAMHM0007</t>
+        </is>
+      </c>
+      <c r="K96" t="n">
+        <v>100000</v>
+      </c>
       <c r="L96" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -11933,12 +12311,16 @@
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="n">
-        <v>0.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I97" t="n">
         <v>4</v>
       </c>
-      <c r="J97" t="inlineStr"/>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>PTOXTAHM0001</t>
+        </is>
+      </c>
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
@@ -11979,12 +12361,16 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>0.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I98" t="n">
         <v>4</v>
       </c>
-      <c r="J98" t="inlineStr"/>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>PTOYAQHM0003</t>
+        </is>
+      </c>
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
@@ -12025,12 +12411,16 @@
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>0.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I99" t="n">
         <v>4</v>
       </c>
-      <c r="J99" t="inlineStr"/>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>PTOYARHM0002</t>
+        </is>
+      </c>
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
@@ -12071,12 +12461,16 @@
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>0.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I100" t="n">
         <v>4</v>
       </c>
-      <c r="J100" t="inlineStr"/>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>PTOYASHM0001</t>
+        </is>
+      </c>
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
@@ -12117,12 +12511,16 @@
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>0.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I101" t="n">
         <v>4</v>
       </c>
-      <c r="J101" t="inlineStr"/>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>PTOYATHM0000</t>
+        </is>
+      </c>
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
@@ -12162,11 +12560,17 @@
         </is>
       </c>
       <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
+      <c r="H102" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I102" t="n">
         <v>4</v>
       </c>
-      <c r="J102" t="inlineStr"/>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>PTOYAUHM0007</t>
+        </is>
+      </c>
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
@@ -12206,11 +12610,17 @@
         </is>
       </c>
       <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
+      <c r="H103" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I103" t="n">
         <v>4</v>
       </c>
-      <c r="J103" t="inlineStr"/>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>PTOYAVHM0006</t>
+        </is>
+      </c>
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
@@ -12250,11 +12660,17 @@
         </is>
       </c>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
+      <c r="H104" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I104" t="n">
         <v>4</v>
       </c>
-      <c r="J104" t="inlineStr"/>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>PTOYAWHM0005</t>
+        </is>
+      </c>
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
@@ -12294,11 +12710,17 @@
         </is>
       </c>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
+      <c r="H105" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I105" t="n">
         <v>4</v>
       </c>
-      <c r="J105" t="inlineStr"/>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>PTOYAXHM0004</t>
+        </is>
+      </c>
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
@@ -12338,11 +12760,17 @@
         </is>
       </c>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
+      <c r="H106" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I106" t="n">
         <v>4</v>
       </c>
-      <c r="J106" t="inlineStr"/>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>PTOXS3HM0000</t>
+        </is>
+      </c>
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
@@ -12382,11 +12810,17 @@
         </is>
       </c>
       <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
+      <c r="H107" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I107" t="n">
         <v>4</v>
       </c>
-      <c r="J107" t="inlineStr"/>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>PTOXS4HM0009</t>
+        </is>
+      </c>
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
@@ -12426,11 +12860,17 @@
         </is>
       </c>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
+      <c r="H108" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I108" t="n">
         <v>4</v>
       </c>
-      <c r="J108" t="inlineStr"/>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>PTOXS5HM0008</t>
+        </is>
+      </c>
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
@@ -12515,13 +12955,19 @@
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I110" t="n">
         <v>4</v>
       </c>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>PTOXTBHM0000</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>2000</v>
+      </c>
       <c r="L110" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -12561,13 +13007,19 @@
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I111" t="n">
         <v>4</v>
       </c>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>PTOYAYHM0003</t>
+        </is>
+      </c>
+      <c r="K111" t="n">
+        <v>2000</v>
+      </c>
       <c r="L111" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -12607,13 +13059,19 @@
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I112" t="n">
         <v>4</v>
       </c>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>PTOYAZHM0002</t>
+        </is>
+      </c>
+      <c r="K112" t="n">
+        <v>2000</v>
+      </c>
       <c r="L112" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -12653,13 +13111,19 @@
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I113" t="n">
         <v>4</v>
       </c>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>PTOYA1HM0008</t>
+        </is>
+      </c>
+      <c r="K113" t="n">
+        <v>2000</v>
+      </c>
       <c r="L113" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -12699,13 +13163,19 @@
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I114" t="n">
         <v>4</v>
       </c>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>PTOYA2HM0007</t>
+        </is>
+      </c>
+      <c r="K114" t="n">
+        <v>2000</v>
+      </c>
       <c r="L114" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -12745,13 +13215,19 @@
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I115" t="n">
         <v>4</v>
       </c>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>PTOYA3HM0006</t>
+        </is>
+      </c>
+      <c r="K115" t="n">
+        <v>2000</v>
+      </c>
       <c r="L115" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -12791,13 +13267,19 @@
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I116" t="n">
         <v>4</v>
       </c>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>PTOYA4HM0005</t>
+        </is>
+      </c>
+      <c r="K116" t="n">
+        <v>2000</v>
+      </c>
       <c r="L116" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -12837,13 +13319,19 @@
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
       <c r="I117" t="n">
         <v>4</v>
       </c>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>PTOYA5HM0004</t>
+        </is>
+      </c>
+      <c r="K117" t="n">
+        <v>2000</v>
+      </c>
       <c r="L117" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -12882,12 +13370,20 @@
         </is>
       </c>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
+      <c r="H118" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I118" t="n">
         <v>4</v>
       </c>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>PTOYA6HM0003</t>
+        </is>
+      </c>
+      <c r="K118" t="n">
+        <v>2000</v>
+      </c>
       <c r="L118" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -12926,12 +13422,20 @@
         </is>
       </c>
       <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
+      <c r="H119" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I119" t="n">
         <v>4</v>
       </c>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>PTOXSMHM0008</t>
+        </is>
+      </c>
+      <c r="K119" t="n">
+        <v>2000</v>
+      </c>
       <c r="L119" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -12970,12 +13474,20 @@
         </is>
       </c>
       <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
+      <c r="H120" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I120" t="n">
         <v>4</v>
       </c>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>PTOXSNHM0007</t>
+        </is>
+      </c>
+      <c r="K120" t="n">
+        <v>2000</v>
+      </c>
       <c r="L120" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -13014,12 +13526,20 @@
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
+      <c r="H121" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I121" t="n">
         <v>4</v>
       </c>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>PTOXSOHM0006</t>
+        </is>
+      </c>
+      <c r="K121" t="n">
+        <v>2000</v>
+      </c>
       <c r="L121" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -13058,12 +13578,20 @@
         </is>
       </c>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
+      <c r="H122" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I122" t="n">
         <v>4</v>
       </c>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>PTOXSPHM0005</t>
+        </is>
+      </c>
+      <c r="K122" t="n">
+        <v>2000</v>
+      </c>
       <c r="L122" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -13102,12 +13630,20 @@
         </is>
       </c>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
+      <c r="H123" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I123" t="n">
         <v>4</v>
       </c>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>PTOXS6HM0007</t>
+        </is>
+      </c>
+      <c r="K123" t="n">
+        <v>2000</v>
+      </c>
       <c r="L123" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -13146,12 +13682,20 @@
         </is>
       </c>
       <c r="G124" t="inlineStr"/>
-      <c r="H124" t="inlineStr"/>
+      <c r="H124" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I124" t="n">
         <v>4</v>
       </c>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>PTOXS7HM0006</t>
+        </is>
+      </c>
+      <c r="K124" t="n">
+        <v>2000</v>
+      </c>
       <c r="L124" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -13190,12 +13734,20 @@
         </is>
       </c>
       <c r="G125" t="inlineStr"/>
-      <c r="H125" t="inlineStr"/>
+      <c r="H125" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I125" t="n">
         <v>4</v>
       </c>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>PTOXS8HM0005</t>
+        </is>
+      </c>
+      <c r="K125" t="n">
+        <v>2000</v>
+      </c>
       <c r="L125" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
@@ -13234,12 +13786,20 @@
         </is>
       </c>
       <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr"/>
+      <c r="H126" t="n">
+        <v>1.06</v>
+      </c>
       <c r="I126" t="n">
         <v>4</v>
       </c>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>PTOXS9HM0004</t>
+        </is>
+      </c>
+      <c r="K126" t="n">
+        <v>2000</v>
+      </c>
       <c r="L126" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>

</xml_diff>

<commit_message>
fix(embed,oxy): texto warning sem '/ 7'; Oxy clip desde 2022-12 + hide EM/EN/EO
- Warning de risco: 'classe 3 vs 6' em vez de 'classe 3 vs 6 / 7' (alinha com
  a decisão anterior de remover '/ 7' da coluna Classe de risco).
- scrapers/oxy.py: corta a série da Google Sheet em 2022-12-21
  (data de constituição do PPR) e rebaseia a 100 nessa data. Assim o
  chart mostra só o histórico real do PPR (40 obs mensais) em vez de
  misturar o track record da estratégia desde 2018.
- Esconde Oxy Cat EM/EN/EO (constavam da CMVM mas não do IFI;
  também não-retail).
</commit_message>
<xml_diff>
--- a/data/ppr_status.xlsx
+++ b/data/ppr_status.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4811,12 +4811,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>smart-invest-ppr-oicvm-moderado-420</t>
+          <t>smart-invest-ppr-oicvm-dinamico-419</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SMART INVEST PPR/OICVM MODERADO</t>
+          <t>SMART INVEST PPR/OICVM DINÂMICO</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4845,7 +4845,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>1.44</v>
+        <v>1.39</v>
       </c>
       <c r="I83" t="n">
         <v>4</v>
@@ -4865,17 +4865,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>fundo-de-investimento-mobiliario-aberto-de-obrigacoes-de-pou-356</t>
+          <t>smart-invest-ppr-oicvm-moderado-420</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Santander Aforro PPR/OICVM</t>
+          <t>SMART INVEST PPR/OICVM MODERADO</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Santander Aforro PPR</t>
+          <t>SMART INVEST PPR</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4895,22 +4895,76 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="H84" t="n">
-        <v>0.88</v>
+        <v>1.44</v>
       </c>
       <c r="I84" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>PTSFFAHM0013</t>
+          <t>PTARMIHM0004</t>
         </is>
       </c>
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
+        <is>
+          <t>FUNDOS DE POUPANÇA-REFORMA HARMONIZADOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>fundo-de-investimento-mobiliario-aberto-de-obrigacoes-de-pou-356</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Santander Aforro PPR/OICVM</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Santander Aforro PPR</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>cmvm</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>historical</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>FI-PPR</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="H85" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="I85" t="n">
+        <v>3</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>PTSFFAHM0013</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr">
         <is>
           <t>FUNDOS DE OBRIGAÇÕES DE FUNDOS POUPANÇA-REFORMA HARMONIZADOS</t>
         </is>
@@ -4927,7 +4981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7863,17 +7917,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>smart-invest-ppr-oicvm-dinamico-419</t>
+          <t>fundo-de-investimento-alternativo-aberto-de-poupanca-reforma-354</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SMART INVEST PPR/OICVM DINÂMICO</t>
+          <t>Santander Poupança Prudente FPR</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SMART INVEST PPR</t>
+          <t>Santander Poupança Prudente</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -7893,33 +7947,37 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>1.39</v>
+        <v>1.34</v>
       </c>
       <c r="I59" t="n">
-        <v>4</v>
-      </c>
-      <c r="J59" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>PTYSAVLM0006</t>
+        </is>
+      </c>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>FUNDOS DE POUPANÇA-REFORMA HARMONIZADOS</t>
+          <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>fundo-de-investimento-alternativo-aberto-de-poupanca-reforma-354</t>
+          <t>fundo-de-investimento-alternativo-aberto-de-poupanca-reforma-355</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Santander Poupança Prudente FPR</t>
+          <t>Santander Poupança Valorização FPR</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Santander Poupança Prudente</t>
+          <t>Santander Poupança Valorização</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -7939,68 +7997,18 @@
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>1.34</v>
+        <v>1.93</v>
       </c>
       <c r="I60" t="n">
         <v>3</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>PTYSAVLM0006</t>
+          <t>PTYMCRLM0006</t>
         </is>
       </c>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
-        <is>
-          <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>fundo-de-investimento-alternativo-aberto-de-poupanca-reforma-355</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Santander Poupança Valorização FPR</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Santander Poupança Valorização</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>cmvm</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>cmvm</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>FI-PPR</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="n">
-        <v>1.93</v>
-      </c>
-      <c r="I61" t="n">
-        <v>3</v>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>PTYMCRLM0006</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr">
         <is>
           <t>FUNDOS DE POUPANÇA-REFORMA NÃO HARMONIZADOS</t>
         </is>
@@ -15301,7 +15309,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>cmvm</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15309,14 +15317,22 @@
           <t>FI-PPR</t>
         </is>
       </c>
-      <c r="G140" t="inlineStr"/>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
       <c r="H140" t="n">
         <v>1.39</v>
       </c>
       <c r="I140" t="n">
         <v>4</v>
       </c>
-      <c r="J140" t="inlineStr"/>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>PTARMIHM0004</t>
+        </is>
+      </c>
       <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr">
         <is>

</xml_diff>